<commit_message>
Implement Steps A-D: Cloud functions config, Android CI/CD build pipeline, E2E walkthrough script, and PDF tax invoice and dispatch challan service
</commit_message>
<xml_diff>
--- a/excel/templates/Pixel_Distributor_Admin.xlsx
+++ b/excel/templates/Pixel_Distributor_Admin.xlsx
@@ -441,7 +441,7 @@
         <v>Last Sync Pull Timestamp</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-09-24T16:20:23.112Z</v>
+        <v>2026-09-24T16:32:32.131Z</v>
       </c>
     </row>
   </sheetData>
@@ -976,7 +976,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-24T16:20:23.108Z</v>
+        <v>2026-09-24T16:32:32.125Z</v>
       </c>
       <c r="B2" t="str">
         <v>admin@pixeldistributor.com</v>

</xml_diff>

<commit_message>
Add production Firebase client SDK with real-time Firestore listeners, Phone OTP service, and Vite environment definitions
</commit_message>
<xml_diff>
--- a/excel/templates/Pixel_Distributor_Admin.xlsx
+++ b/excel/templates/Pixel_Distributor_Admin.xlsx
@@ -441,7 +441,7 @@
         <v>Last Sync Pull Timestamp</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-09-24T16:32:32.131Z</v>
+        <v>2026-09-24T16:56:51.826Z</v>
       </c>
     </row>
   </sheetData>
@@ -976,7 +976,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-24T16:32:32.125Z</v>
+        <v>2026-09-24T16:56:51.821Z</v>
       </c>
       <c r="B2" t="str">
         <v>admin@pixeldistributor.com</v>

</xml_diff>

<commit_message>
Configure live Firebase project pixel-distributor with Firestore seeding script, Phone OTP auth modal, and real-time document listeners
</commit_message>
<xml_diff>
--- a/excel/templates/Pixel_Distributor_Admin.xlsx
+++ b/excel/templates/Pixel_Distributor_Admin.xlsx
@@ -441,7 +441,7 @@
         <v>Last Sync Pull Timestamp</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-09-24T16:56:51.826Z</v>
+        <v>2026-09-24T17:26:44.141Z</v>
       </c>
     </row>
   </sheetData>
@@ -976,7 +976,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-24T16:56:51.821Z</v>
+        <v>2026-09-24T17:26:44.124Z</v>
       </c>
       <c r="B2" t="str">
         <v>admin@pixeldistributor.com</v>

</xml_diff>

<commit_message>
Transition to Plan A: Excel-First Administration, Direct Cloud Firestore Sync Engine, and Chameleon Dealer Mobile PWA
</commit_message>
<xml_diff>
--- a/excel/templates/Pixel_Distributor_Admin.xlsx
+++ b/excel/templates/Pixel_Distributor_Admin.xlsx
@@ -6,8 +6,8 @@
     <sheet name="DASHBOARD" sheetId="1" r:id="rId1"/>
     <sheet name="DEALER_MASTER" sheetId="2" r:id="rId2"/>
     <sheet name="PRODUCT_MASTER" sheetId="3" r:id="rId3"/>
-    <sheet name="INVENTORY" sheetId="4" r:id="rId4"/>
-    <sheet name="ORDERS" sheetId="5" r:id="rId5"/>
+    <sheet name="INVENTORY_BALANCES" sheetId="4" r:id="rId4"/>
+    <sheet name="PURCHASE_ORDERS" sheetId="5" r:id="rId5"/>
     <sheet name="ACTIVITY_LOG" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -414,39 +414,55 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Total Active Dealers</v>
-      </c>
-      <c r="B2">
-        <v>3</v>
+        <v>Platform Mode</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Plan A: Excel-First Administration</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Total Catalog SKUs</v>
-      </c>
-      <c r="B3">
-        <v>3</v>
+        <v>Cloud Database</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Google Cloud Firestore (pixel-distributor)</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Total Orders Captured</v>
+        <v>Total Active Dealers</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Total Catalog SKUs</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Total Orders Captured</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
         <v>Last Sync Pull Timestamp</v>
       </c>
-      <c r="B5" t="str">
-        <v>2026-09-24T17:26:44.141Z</v>
+      <c r="B7" t="str">
+        <v>2026-09-24T18:07:42.222Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -976,10 +992,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-24T17:26:44.124Z</v>
+        <v>2026-09-24T18:07:42.210Z</v>
       </c>
       <c r="B2" t="str">
-        <v>admin@pixeldistributor.com</v>
+        <v>naren7703@gmail.com</v>
       </c>
       <c r="C2" t="str">
         <v>EXCEL_SYNC_PUSH_EXECUTED</v>

</xml_diff>